<commit_message>
print bad to screen
</commit_message>
<xml_diff>
--- a/machine_learning/injection/DDLUCJ-experiment-pipeline/trash.xlsx
+++ b/machine_learning/injection/DDLUCJ-experiment-pipeline/trash.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,20 +466,15 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>Energy (HCI)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Energy (HCI)</t>
+          <t>Energy (HF)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Energy (HF)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Energy (CASCI)</t>
         </is>
@@ -519,15 +514,12 @@
         <v>10</v>
       </c>
       <c r="I2" t="n">
-        <v>-28665435.73824892</v>
+        <v>-154.9179424757513</v>
       </c>
       <c r="J2" t="n">
-        <v>-154.9179424757513</v>
-      </c>
-      <c r="K2" t="n">
         <v>-154.9167852198248</v>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -563,15 +555,12 @@
         <v>10</v>
       </c>
       <c r="I3" t="n">
-        <v>-57284904.59216711</v>
+        <v>-154.9506284389599</v>
       </c>
       <c r="J3" t="n">
-        <v>-154.9506284389599</v>
-      </c>
-      <c r="K3" t="n">
         <v>-154.9399130373333</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -601,34 +590,31 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>-138011.419486301</v>
+        <v>-171609.2046135756</v>
       </c>
       <c r="H4" t="n">
         <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>-137674606.6030501</v>
+        <v>-336.8128832509636</v>
       </c>
       <c r="J4" t="n">
-        <v>-336.8128832509636</v>
-      </c>
-      <c r="K4" t="n">
         <v>-336.812789763256</v>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>STO-3G</t>
+          <t>aug-cc-pVDZ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>prop-2-en-1-ol</t>
+          <t>buta-1,3-diene</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -641,161 +627,149 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MP2</t>
+          <t>CCSD</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>-86107.21411246741</v>
+        <v>-64449.17383315753</v>
       </c>
       <c r="H5" t="n">
         <v>10</v>
       </c>
       <c r="I5" t="n">
-        <v>-85917487.0967143</v>
+        <v>-154.9506284389599</v>
       </c>
       <c r="J5" t="n">
-        <v>-189.7270157531005</v>
-      </c>
-      <c r="K5" t="n">
-        <v>-189.4804271888057</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
+        <v>-154.9399130373333</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>aug-cc-pVDZ</t>
+          <t>STO-3G</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>buta-1,3-diene</t>
+          <t>prop-2-en-1-ol</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LUCJ(L=3)</t>
+          <t>LUCJ(L=2)</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CCSD</t>
+          <t>random</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>-64449.17383315753</v>
+        <v>-102438.5962274746</v>
       </c>
       <c r="H6" t="n">
         <v>10</v>
       </c>
       <c r="I6" t="n">
-        <v>-64294223.20471857</v>
+        <v>-189.7270157531005</v>
       </c>
       <c r="J6" t="n">
-        <v>-154.9506284389599</v>
-      </c>
-      <c r="K6" t="n">
-        <v>-154.9399130373333</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
+        <v>-189.4804271888057</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>380</v>
+        <v>397</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>STO-3G</t>
+          <t>cc-pVDZ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>prop-2-en-1-ol</t>
+          <t>fluoroform</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LUCJ(L=2)</t>
+          <t>LUCJ(L=1)</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>random</t>
+          <t>ML_exact</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>-95920.92593647477</v>
+        <v>-105440.3491046589</v>
       </c>
       <c r="H7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I7" t="n">
-        <v>-95731198.92072167</v>
+        <v>-336.8244320005772</v>
       </c>
       <c r="J7" t="n">
-        <v>-189.7270157531005</v>
-      </c>
-      <c r="K7" t="n">
-        <v>-189.4804271888057</v>
-      </c>
-      <c r="L7" t="inlineStr"/>
+        <v>-336.7867835322212</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>397</v>
+        <v>434</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>cc-pVDZ</t>
+          <t>aug-cc-pVDZ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>fluoroform</t>
+          <t>(Z)-1-fluoroprop-1-ene</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>LUCJ(L=1)</t>
+          <t>LUCJ(L=2)</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ML_exact</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>-153852.6384371886</v>
+        <v>-82689.37866547176</v>
       </c>
       <c r="H8" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I8" t="n">
-        <v>-153515814.005188</v>
+        <v>-215.950411541533</v>
       </c>
       <c r="J8" t="n">
-        <v>-336.8244320005772</v>
-      </c>
-      <c r="K8" t="n">
-        <v>-336.7867835322212</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
+        <v>-215.9496895929251</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>416</v>
+        <v>535</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -804,42 +778,39 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>prop-2-en-1-ol</t>
+          <t>(Z)-1-fluoroprop-1-ene</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LUCJ(L=5)</t>
+          <t>LUCJ(L=3)</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>random</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>-69745.38585778153</v>
+        <v>-25477.33493414854</v>
       </c>
       <c r="H9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I9" t="n">
-        <v>-69553432.08581606</v>
+        <v>-215.950411541533</v>
       </c>
       <c r="J9" t="n">
-        <v>-191.9537719654783</v>
-      </c>
-      <c r="K9" t="n">
-        <v>-191.9516344755187</v>
-      </c>
-      <c r="L9" t="inlineStr"/>
+        <v>-215.9496895929251</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>434</v>
+        <v>561</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -848,46 +819,43 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
+          <t>prop-2-en-1-ol</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>LUCJ(L=2)</t>
+          <t>LUCJ(L=5)</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ML_exact</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>-65105.91137328053</v>
+        <v>-58372.75649593984</v>
       </c>
       <c r="H10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I10" t="n">
-        <v>-64889960.961739</v>
+        <v>-191.9537719654783</v>
       </c>
       <c r="J10" t="n">
-        <v>-215.950411541533</v>
-      </c>
-      <c r="K10" t="n">
-        <v>-215.9496895929251</v>
-      </c>
-      <c r="L10" t="inlineStr"/>
+        <v>-191.9516344755187</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>459</v>
+        <v>681</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>STO-3G</t>
+          <t>aug-cc-pVDZ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -897,85 +865,79 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LUCJ(L=4)</t>
+          <t>LUCJ(L=3)</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>random</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>-43361.06128316602</v>
+        <v>-34155.39003418432</v>
       </c>
       <c r="H11" t="n">
         <v>9</v>
       </c>
       <c r="I11" t="n">
-        <v>-43147717.66935617</v>
+        <v>-215.950411541533</v>
       </c>
       <c r="J11" t="n">
-        <v>-213.3436138098513</v>
-      </c>
-      <c r="K11" t="n">
-        <v>-213.1164694544959</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
+        <v>-215.9496895929251</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>535</v>
+        <v>884</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>aug-cc-pVDZ</t>
+          <t>STO-3G</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
+          <t>fluoroform</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LUCJ(L=3)</t>
+          <t>LUCJ(L=1)</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>CCSD</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>-66861.83224124661</v>
+        <v>-109290.3703035947</v>
       </c>
       <c r="H12" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I12" t="n">
-        <v>-66645881.82970507</v>
+        <v>-332.2216949700667</v>
       </c>
       <c r="J12" t="n">
-        <v>-215.950411541533</v>
-      </c>
-      <c r="K12" t="n">
-        <v>-215.9496895929251</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
+        <v>-332.0975924899263</v>
+      </c>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>561</v>
+        <v>1032</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>aug-cc-pVDZ</t>
+          <t>STO-3G</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -985,517 +947,71 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>LUCJ(L=5)</t>
+          <t>LUCJ(L=2)</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ML_exact</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>-34609.32442347352</v>
+        <v>-80031.22170701248</v>
       </c>
       <c r="H13" t="n">
         <v>10</v>
       </c>
       <c r="I13" t="n">
-        <v>-34417370.65150805</v>
+        <v>-189.7270157531005</v>
       </c>
       <c r="J13" t="n">
-        <v>-191.9537719654783</v>
-      </c>
-      <c r="K13" t="n">
-        <v>-191.9516344755187</v>
-      </c>
-      <c r="L13" t="inlineStr"/>
+        <v>-189.4804271888057</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>613</v>
+        <v>1036</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>cc-pVDZ</t>
+          <t>aug-cc-pVDZ</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>prop-2-en-1-ol</t>
+          <t>buta-1,3-diene</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>LUCJ(L=3)</t>
+          <t>LUCJ(L=1)</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>CCSD</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>-77926.65815326312</v>
+        <v>-70646.0604888675</v>
       </c>
       <c r="H14" t="n">
         <v>10</v>
       </c>
       <c r="I14" t="n">
-        <v>-77734660.67237608</v>
+        <v>-154.9506284389599</v>
       </c>
       <c r="J14" t="n">
-        <v>-191.9974808870427</v>
-      </c>
-      <c r="K14" t="n">
-        <v>-191.9364953941601</v>
-      </c>
-      <c r="L14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>654</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>prop-2-en-1-ol</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>LUCJ(L=5)</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>5</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>ML_exact</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>-80044.31217606291</v>
-      </c>
-      <c r="H15" t="n">
-        <v>10</v>
-      </c>
-      <c r="I15" t="n">
-        <v>-79852314.69517587</v>
-      </c>
-      <c r="J15" t="n">
-        <v>-191.9974808870427</v>
-      </c>
-      <c r="K15" t="n">
-        <v>-191.9364953941601</v>
-      </c>
-      <c r="L15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>681</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>aug-cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>LUCJ(L=3)</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>-53818.86718026046</v>
-      </c>
-      <c r="H16" t="n">
-        <v>9</v>
-      </c>
-      <c r="I16" t="n">
-        <v>-53602916.76871893</v>
-      </c>
-      <c r="J16" t="n">
-        <v>-215.950411541533</v>
-      </c>
-      <c r="K16" t="n">
-        <v>-215.9496895929251</v>
-      </c>
-      <c r="L16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>756</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>aug-cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>LUCJ(L=4)</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>-59927.74991335726</v>
-      </c>
-      <c r="H17" t="n">
-        <v>9</v>
-      </c>
-      <c r="I17" t="n">
-        <v>-59711799.50181573</v>
-      </c>
-      <c r="J17" t="n">
-        <v>-215.950411541533</v>
-      </c>
-      <c r="K17" t="n">
-        <v>-215.9496895929251</v>
-      </c>
-      <c r="L17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>823</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>aug-cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>LUCJ(L=1)</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>ML_exact</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>-90136.87670158829</v>
-      </c>
-      <c r="H18" t="n">
-        <v>9</v>
-      </c>
-      <c r="I18" t="n">
-        <v>-89920926.29004675</v>
-      </c>
-      <c r="J18" t="n">
-        <v>-215.950411541533</v>
-      </c>
-      <c r="K18" t="n">
-        <v>-215.9496895929251</v>
-      </c>
-      <c r="L18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>884</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>STO-3G</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>fluoroform</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>LUCJ(L=1)</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>CCSD</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>-23390.63027026573</v>
-      </c>
-      <c r="H19" t="n">
-        <v>5</v>
-      </c>
-      <c r="I19" t="n">
-        <v>-23058408.57529566</v>
-      </c>
-      <c r="J19" t="n">
-        <v>-332.2216949700667</v>
-      </c>
-      <c r="K19" t="n">
-        <v>-332.0975924899263</v>
-      </c>
-      <c r="L19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>927</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>LUCJ(L=4)</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>-88821.6776168841</v>
-      </c>
-      <c r="H20" t="n">
-        <v>9</v>
-      </c>
-      <c r="I20" t="n">
-        <v>-88605679.5982264</v>
-      </c>
-      <c r="J20" t="n">
-        <v>-215.9980186576996</v>
-      </c>
-      <c r="K20" t="n">
-        <v>-215.9369612176939</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>1020</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>but-1-yne</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>LUCJ(L=3)</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>MP2</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>-47980.07241711803</v>
-      </c>
-      <c r="H21" t="n">
-        <v>10</v>
-      </c>
-      <c r="I21" t="n">
-        <v>-47825071.96875379</v>
-      </c>
-      <c r="J21" t="n">
-        <v>-155.0004483642394</v>
-      </c>
-      <c r="K21" t="n">
-        <v>-154.9113882737664</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>1032</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>STO-3G</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>prop-2-en-1-ol</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>LUCJ(L=2)</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>-20541.60368971845</v>
-      </c>
-      <c r="H22" t="n">
-        <v>10</v>
-      </c>
-      <c r="I22" t="n">
-        <v>-20351876.67396534</v>
-      </c>
-      <c r="J22" t="n">
-        <v>-189.7270157531005</v>
-      </c>
-      <c r="K22" t="n">
-        <v>-189.4804271888057</v>
-      </c>
-      <c r="L22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>1036</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>aug-cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>buta-1,3-diene</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>LUCJ(L=1)</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>CCSD</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>-78696.50371377631</v>
-      </c>
-      <c r="H23" t="n">
-        <v>10</v>
-      </c>
-      <c r="I23" t="n">
-        <v>-78541553.08533736</v>
-      </c>
-      <c r="J23" t="n">
-        <v>-154.9506284389599</v>
-      </c>
-      <c r="K23" t="n">
         <v>-154.9399130373333</v>
       </c>
-      <c r="L23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>1043</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>LUCJ(L=2)</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>CCSD</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>-24562.86904081846</v>
-      </c>
-      <c r="H24" t="n">
-        <v>9</v>
-      </c>
-      <c r="I24" t="n">
-        <v>-24346871.02216076</v>
-      </c>
-      <c r="J24" t="n">
-        <v>-215.9980186576996</v>
-      </c>
-      <c r="K24" t="n">
-        <v>-215.9369612176939</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Thu 16 Apr 2026 10:57:33 EDT
</commit_message>
<xml_diff>
--- a/machine_learning/injection/DDLUCJ-experiment-pipeline/trash.xlsx
+++ b/machine_learning/injection/DDLUCJ-experiment-pipeline/trash.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,7 +482,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>35</v>
+        <v>187</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -491,48 +491,48 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>but-1-yne</t>
+          <t>fluoroform</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LUCJ(L=5)</t>
+          <t>LUCJ(L=1)</t>
         </is>
       </c>
       <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ML_exact</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>-153259.0435841685</v>
+      </c>
+      <c r="H2" t="n">
         <v>5</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>-28820.35368072467</v>
-      </c>
-      <c r="H2" t="n">
-        <v>10</v>
-      </c>
       <c r="I2" t="n">
-        <v>-154.9179424757513</v>
+        <v>-336.8128832509636</v>
       </c>
       <c r="J2" t="n">
-        <v>-154.9167852198248</v>
+        <v>-336.812789763256</v>
       </c>
       <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>81</v>
+        <v>397</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aug-cc-pVDZ</t>
+          <t>cc-pVDZ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>buta-1,3-diene</t>
+          <t>fluoroform</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -545,26 +545,26 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>random</t>
+          <t>ML_exact</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>-57439.85522060606</v>
+        <v>-153676.1555048768</v>
       </c>
       <c r="H3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I3" t="n">
-        <v>-154.9506284389599</v>
+        <v>-336.8244320005772</v>
       </c>
       <c r="J3" t="n">
-        <v>-154.9399130373333</v>
+        <v>-336.7867835322212</v>
       </c>
       <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>187</v>
+        <v>434</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -573,39 +573,39 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>fluoroform</t>
+          <t>(Z)-1-fluoroprop-1-ene</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>LUCJ(L=1)</t>
+          <t>LUCJ(L=2)</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ML_exact</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>-171609.2046135756</v>
+        <v>-82689.37866547176</v>
       </c>
       <c r="H4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I4" t="n">
-        <v>-336.8128832509636</v>
+        <v>-215.950411541533</v>
       </c>
       <c r="J4" t="n">
-        <v>-336.812789763256</v>
+        <v>-215.9496895929251</v>
       </c>
       <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>368</v>
+        <v>561</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -614,57 +614,57 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>buta-1,3-diene</t>
+          <t>prop-2-en-1-ol</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LUCJ(L=3)</t>
+          <t>LUCJ(L=5)</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CCSD</t>
+          <t>ML_exact</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>-64449.17383315753</v>
+        <v>-25006.80731456201</v>
       </c>
       <c r="H5" t="n">
         <v>10</v>
       </c>
       <c r="I5" t="n">
-        <v>-154.9506284389599</v>
+        <v>-191.9537719654783</v>
       </c>
       <c r="J5" t="n">
-        <v>-154.9399130373333</v>
+        <v>-191.9516344755187</v>
       </c>
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>380</v>
+        <v>681</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>STO-3G</t>
+          <t>aug-cc-pVDZ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>prop-2-en-1-ol</t>
+          <t>(Z)-1-fluoroprop-1-ene</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LUCJ(L=2)</t>
+          <t>LUCJ(L=3)</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -672,26 +672,26 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>-102438.5962274746</v>
+        <v>-52922.37172517645</v>
       </c>
       <c r="H6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I6" t="n">
-        <v>-189.7270157531005</v>
+        <v>-215.950411541533</v>
       </c>
       <c r="J6" t="n">
-        <v>-189.4804271888057</v>
+        <v>-215.9496895929251</v>
       </c>
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>397</v>
+        <v>884</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>cc-pVDZ</t>
+          <t>STO-3G</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -709,35 +709,35 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ML_exact</t>
+          <t>CCSD</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>-105440.3491046589</v>
+        <v>-106137.1323894411</v>
       </c>
       <c r="H7" t="n">
         <v>5</v>
       </c>
       <c r="I7" t="n">
-        <v>-336.8244320005772</v>
+        <v>-332.2216949700667</v>
       </c>
       <c r="J7" t="n">
-        <v>-336.7867835322212</v>
+        <v>-332.0975924899263</v>
       </c>
       <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>434</v>
+        <v>1032</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>aug-cc-pVDZ</t>
+          <t>STO-3G</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
+          <t>prop-2-en-1-ol</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -754,22 +754,22 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>-82689.37866547176</v>
+        <v>-85312.39850706911</v>
       </c>
       <c r="H8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I8" t="n">
-        <v>-215.950411541533</v>
+        <v>-189.7270157531005</v>
       </c>
       <c r="J8" t="n">
-        <v>-215.9496895929251</v>
+        <v>-189.4804271888057</v>
       </c>
       <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>535</v>
+        <v>1036</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -778,240 +778,35 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
+          <t>buta-1,3-diene</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LUCJ(L=3)</t>
+          <t>LUCJ(L=1)</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>CCSD</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>-25477.33493414854</v>
+        <v>-58430.16994785824</v>
       </c>
       <c r="H9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I9" t="n">
-        <v>-215.950411541533</v>
+        <v>-154.9506284389599</v>
       </c>
       <c r="J9" t="n">
-        <v>-215.9496895929251</v>
+        <v>-154.9399130373333</v>
       </c>
       <c r="K9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>561</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>aug-cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>prop-2-en-1-ol</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>LUCJ(L=5)</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>ML_exact</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>-58372.75649593984</v>
-      </c>
-      <c r="H10" t="n">
-        <v>10</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-191.9537719654783</v>
-      </c>
-      <c r="J10" t="n">
-        <v>-191.9516344755187</v>
-      </c>
-      <c r="K10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>681</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>aug-cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>LUCJ(L=3)</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>-34155.39003418432</v>
-      </c>
-      <c r="H11" t="n">
-        <v>9</v>
-      </c>
-      <c r="I11" t="n">
-        <v>-215.950411541533</v>
-      </c>
-      <c r="J11" t="n">
-        <v>-215.9496895929251</v>
-      </c>
-      <c r="K11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>884</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>STO-3G</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>fluoroform</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>LUCJ(L=1)</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>CCSD</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>-109290.3703035947</v>
-      </c>
-      <c r="H12" t="n">
-        <v>5</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-332.2216949700667</v>
-      </c>
-      <c r="J12" t="n">
-        <v>-332.0975924899263</v>
-      </c>
-      <c r="K12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>1032</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>STO-3G</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>prop-2-en-1-ol</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>LUCJ(L=2)</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>-80031.22170701248</v>
-      </c>
-      <c r="H13" t="n">
-        <v>10</v>
-      </c>
-      <c r="I13" t="n">
-        <v>-189.7270157531005</v>
-      </c>
-      <c r="J13" t="n">
-        <v>-189.4804271888057</v>
-      </c>
-      <c r="K13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>1036</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>aug-cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>buta-1,3-diene</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>LUCJ(L=1)</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>CCSD</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>-70646.0604888675</v>
-      </c>
-      <c r="H14" t="n">
-        <v>10</v>
-      </c>
-      <c r="I14" t="n">
-        <v>-154.9506284389599</v>
-      </c>
-      <c r="J14" t="n">
-        <v>-154.9399130373333</v>
-      </c>
-      <c r="K14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fri 17 Apr 2026 17:18:48 EDT
</commit_message>
<xml_diff>
--- a/machine_learning/injection/DDLUCJ-experiment-pipeline/trash.xlsx
+++ b/machine_learning/injection/DDLUCJ-experiment-pipeline/trash.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,48 +605,48 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>561</v>
+        <v>884</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>aug-cc-pVDZ</t>
+          <t>STO-3G</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>prop-2-en-1-ol</t>
+          <t>fluoroform</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LUCJ(L=5)</t>
+          <t>LUCJ(L=1)</t>
         </is>
       </c>
       <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CCSD</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>-106137.1323894411</v>
+      </c>
+      <c r="H5" t="n">
         <v>5</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>ML_exact</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>-25006.80731456201</v>
-      </c>
-      <c r="H5" t="n">
-        <v>10</v>
-      </c>
       <c r="I5" t="n">
-        <v>-191.9537719654783</v>
+        <v>-332.2216949700667</v>
       </c>
       <c r="J5" t="n">
-        <v>-191.9516344755187</v>
+        <v>-332.0975924899263</v>
       </c>
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>681</v>
+        <v>1036</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -655,158 +655,35 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>(Z)-1-fluoroprop-1-ene</t>
+          <t>buta-1,3-diene</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LUCJ(L=3)</t>
+          <t>LUCJ(L=1)</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>random</t>
+          <t>CCSD</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>-52922.37172517645</v>
+        <v>-58430.16994785824</v>
       </c>
       <c r="H6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I6" t="n">
-        <v>-215.950411541533</v>
+        <v>-154.9506284389599</v>
       </c>
       <c r="J6" t="n">
-        <v>-215.9496895929251</v>
+        <v>-154.9399130373333</v>
       </c>
       <c r="K6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>884</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>STO-3G</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>fluoroform</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>LUCJ(L=1)</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>CCSD</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>-106137.1323894411</v>
-      </c>
-      <c r="H7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-332.2216949700667</v>
-      </c>
-      <c r="J7" t="n">
-        <v>-332.0975924899263</v>
-      </c>
-      <c r="K7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>1032</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>STO-3G</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>prop-2-en-1-ol</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>LUCJ(L=2)</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>-85312.39850706911</v>
-      </c>
-      <c r="H8" t="n">
-        <v>10</v>
-      </c>
-      <c r="I8" t="n">
-        <v>-189.7270157531005</v>
-      </c>
-      <c r="J8" t="n">
-        <v>-189.4804271888057</v>
-      </c>
-      <c r="K8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>1036</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>aug-cc-pVDZ</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>buta-1,3-diene</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>LUCJ(L=1)</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>CCSD</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>-58430.16994785824</v>
-      </c>
-      <c r="H9" t="n">
-        <v>10</v>
-      </c>
-      <c r="I9" t="n">
-        <v>-154.9506284389599</v>
-      </c>
-      <c r="J9" t="n">
-        <v>-154.9399130373333</v>
-      </c>
-      <c r="K9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>